<commit_message>
feat: Carga automatica desde red Q:\005 - Prenomina\Reloj e importacion de asistencias de agosto (12 al 26 de agosto)
</commit_message>
<xml_diff>
--- a/asistencias/historico_semanal.xlsx
+++ b/asistencias/historico_semanal.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="96">
   <si>
     <t>Semana</t>
   </si>
@@ -76,6 +76,15 @@
     <t>Semana 31</t>
   </si>
   <si>
+    <t>Semana 33</t>
+  </si>
+  <si>
+    <t>Semana 34</t>
+  </si>
+  <si>
+    <t>Semana 35</t>
+  </si>
+  <si>
     <t>05-may-26</t>
   </si>
   <si>
@@ -115,6 +124,15 @@
     <t>27-jul-26</t>
   </si>
   <si>
+    <t>12-aug-26</t>
+  </si>
+  <si>
+    <t>17-aug-26</t>
+  </si>
+  <si>
+    <t>24-aug-26</t>
+  </si>
+  <si>
     <t>08-may-26</t>
   </si>
   <si>
@@ -154,6 +172,15 @@
     <t>31-jul-26</t>
   </si>
   <si>
+    <t>14-aug-26</t>
+  </si>
+  <si>
+    <t>21-aug-26</t>
+  </si>
+  <si>
+    <t>26-aug-26</t>
+  </si>
+  <si>
     <t>68.57% (24 de 35)</t>
   </si>
   <si>
@@ -184,6 +211,15 @@
     <t>86.15% (56 de 65)</t>
   </si>
   <si>
+    <t>73.08% (19 de 26)</t>
+  </si>
+  <si>
+    <t>80.00% (52 de 65)</t>
+  </si>
+  <si>
+    <t>82.05% (32 de 39)</t>
+  </si>
+  <si>
     <t>66.67% (16 de 24)</t>
   </si>
   <si>
@@ -220,6 +256,15 @@
     <t>64.91% (37 de 57)</t>
   </si>
   <si>
+    <t>63.16% (12 de 19)</t>
+  </si>
+  <si>
+    <t>53.85% (28 de 52)</t>
+  </si>
+  <si>
+    <t>50.00% (16 de 32)</t>
+  </si>
+  <si>
     <t>31.43% (11 de 35)</t>
   </si>
   <si>
@@ -248,6 +293,15 @@
   </si>
   <si>
     <t>13.85% (9 de 65)</t>
+  </si>
+  <si>
+    <t>26.92% (7 de 26)</t>
+  </si>
+  <si>
+    <t>20.00% (13 de 65)</t>
+  </si>
+  <si>
+    <t>17.95% (7 de 39)</t>
   </si>
 </sst>
 </file>
@@ -579,7 +633,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -613,19 +667,19 @@
         <v>2026</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D2" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="E2" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="F2" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="G2" t="s">
-        <v>68</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -636,19 +690,19 @@
         <v>2026</v>
       </c>
       <c r="C3" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D3" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="E3" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="F3" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="G3" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -659,19 +713,19 @@
         <v>2026</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D4" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="E4" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="F4" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="G4" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -682,19 +736,19 @@
         <v>2026</v>
       </c>
       <c r="C5" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="D5" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="E5" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="F5" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="G5" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -705,19 +759,19 @@
         <v>2026</v>
       </c>
       <c r="C6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D6" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="E6" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="F6" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="G6" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -728,19 +782,19 @@
         <v>2026</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D7" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="E7" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="F7" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="G7" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -751,19 +805,19 @@
         <v>2026</v>
       </c>
       <c r="C8" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D8" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="E8" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="F8" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="G8" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -774,19 +828,19 @@
         <v>2026</v>
       </c>
       <c r="C9" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D9" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="E9" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="F9" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="G9" t="s">
-        <v>74</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -797,19 +851,19 @@
         <v>2026</v>
       </c>
       <c r="C10" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D10" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="E10" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="F10" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="G10" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -820,19 +874,19 @@
         <v>2026</v>
       </c>
       <c r="C11" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D11" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="E11" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="F11" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="G11" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -843,19 +897,19 @@
         <v>2026</v>
       </c>
       <c r="C12" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D12" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="E12" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="F12" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="G12" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -866,19 +920,19 @@
         <v>2026</v>
       </c>
       <c r="C13" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D13" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E13" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="F13" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="G13" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -889,19 +943,88 @@
         <v>2026</v>
       </c>
       <c r="C14" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D14" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="E14" t="s">
+        <v>63</v>
+      </c>
+      <c r="F14" t="s">
+        <v>79</v>
+      </c>
+      <c r="G14" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15">
+        <v>2026</v>
+      </c>
+      <c r="C15" t="s">
+        <v>36</v>
+      </c>
+      <c r="D15" t="s">
+        <v>52</v>
+      </c>
+      <c r="E15" t="s">
+        <v>65</v>
+      </c>
+      <c r="F15" t="s">
+        <v>80</v>
+      </c>
+      <c r="G15" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16">
+        <v>2026</v>
+      </c>
+      <c r="C16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D16" t="s">
+        <v>53</v>
+      </c>
+      <c r="E16" t="s">
+        <v>66</v>
+      </c>
+      <c r="F16" t="s">
+        <v>81</v>
+      </c>
+      <c r="G16" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17">
+        <v>2026</v>
+      </c>
+      <c r="C17" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" t="s">
         <v>54</v>
       </c>
-      <c r="F14" t="s">
+      <c r="E17" t="s">
         <v>67</v>
       </c>
-      <c r="G14" t="s">
-        <v>76</v>
+      <c r="F17" t="s">
+        <v>82</v>
+      </c>
+      <c r="G17" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Importacion completa de archivos de asistencia de agosto (3 al 26 de agosto) y soporte multiruta local (Q: y Google Drive)
</commit_message>
<xml_diff>
--- a/asistencias/historico_semanal.xlsx
+++ b/asistencias/historico_semanal.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="98">
   <si>
     <t>Semana</t>
   </si>
@@ -76,6 +76,9 @@
     <t>Semana 31</t>
   </si>
   <si>
+    <t>Semana 32</t>
+  </si>
+  <si>
     <t>Semana 33</t>
   </si>
   <si>
@@ -124,7 +127,10 @@
     <t>27-jul-26</t>
   </si>
   <si>
-    <t>12-aug-26</t>
+    <t>03-aug-26</t>
+  </si>
+  <si>
+    <t>10-aug-26</t>
   </si>
   <si>
     <t>17-aug-26</t>
@@ -172,6 +178,9 @@
     <t>31-jul-26</t>
   </si>
   <si>
+    <t>07-aug-26</t>
+  </si>
+  <si>
     <t>14-aug-26</t>
   </si>
   <si>
@@ -211,9 +220,6 @@
     <t>86.15% (56 de 65)</t>
   </si>
   <si>
-    <t>73.08% (19 de 26)</t>
-  </si>
-  <si>
     <t>80.00% (52 de 65)</t>
   </si>
   <si>
@@ -256,7 +262,10 @@
     <t>64.91% (37 de 57)</t>
   </si>
   <si>
-    <t>63.16% (12 de 19)</t>
+    <t>53.57% (30 de 56)</t>
+  </si>
+  <si>
+    <t>59.62% (31 de 52)</t>
   </si>
   <si>
     <t>53.85% (28 de 52)</t>
@@ -293,9 +302,6 @@
   </si>
   <si>
     <t>13.85% (9 de 65)</t>
-  </si>
-  <si>
-    <t>26.92% (7 de 26)</t>
   </si>
   <si>
     <t>20.00% (13 de 65)</t>
@@ -633,7 +639,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -667,19 +673,19 @@
         <v>2026</v>
       </c>
       <c r="C2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="F2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G2" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -690,19 +696,19 @@
         <v>2026</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D3" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E3" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="F3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -713,19 +719,19 @@
         <v>2026</v>
       </c>
       <c r="C4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -736,19 +742,19 @@
         <v>2026</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E5" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="F5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G5" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -759,19 +765,19 @@
         <v>2026</v>
       </c>
       <c r="C6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E6" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="F6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G6" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -782,19 +788,19 @@
         <v>2026</v>
       </c>
       <c r="C7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E7" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="F7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G7" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -805,19 +811,19 @@
         <v>2026</v>
       </c>
       <c r="C8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E8" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="F8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G8" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -828,19 +834,19 @@
         <v>2026</v>
       </c>
       <c r="C9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E9" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="F9" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G9" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -851,19 +857,19 @@
         <v>2026</v>
       </c>
       <c r="C10" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E10" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F10" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G10" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -874,19 +880,19 @@
         <v>2026</v>
       </c>
       <c r="C11" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D11" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E11" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="F11" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G11" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -897,19 +903,19 @@
         <v>2026</v>
       </c>
       <c r="C12" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D12" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E12" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F12" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G12" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -920,19 +926,19 @@
         <v>2026</v>
       </c>
       <c r="C13" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D13" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E13" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="F13" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G13" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -943,19 +949,19 @@
         <v>2026</v>
       </c>
       <c r="C14" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D14" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E14" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="F14" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G14" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -966,19 +972,19 @@
         <v>2026</v>
       </c>
       <c r="C15" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D15" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F15" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G15" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -989,19 +995,19 @@
         <v>2026</v>
       </c>
       <c r="C16" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D16" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F16" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G16" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -1012,19 +1018,42 @@
         <v>2026</v>
       </c>
       <c r="C17" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D17" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F17" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G17" t="s">
-        <v>95</v>
+        <v>96</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18">
+        <v>2026</v>
+      </c>
+      <c r="C18" t="s">
+        <v>40</v>
+      </c>
+      <c r="D18" t="s">
+        <v>57</v>
+      </c>
+      <c r="E18" t="s">
+        <v>69</v>
+      </c>
+      <c r="F18" t="s">
+        <v>85</v>
+      </c>
+      <c r="G18" t="s">
+        <v>97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Agregar ruta automatica Q:\005 - RH\Reloj e importar asistencias de septiembre (1 al 8 de septiembre)
</commit_message>
<xml_diff>
--- a/asistencias/historico_semanal.xlsx
+++ b/asistencias/historico_semanal.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="110">
   <si>
     <t>Semana</t>
   </si>
@@ -88,6 +88,12 @@
     <t>Semana 35</t>
   </si>
   <si>
+    <t>Semana 36</t>
+  </si>
+  <si>
+    <t>Semana 37</t>
+  </si>
+  <si>
     <t>05-may-26</t>
   </si>
   <si>
@@ -139,6 +145,12 @@
     <t>24-aug-26</t>
   </si>
   <si>
+    <t>01-sep-26</t>
+  </si>
+  <si>
+    <t>07-sep-26</t>
+  </si>
+  <si>
     <t>08-may-26</t>
   </si>
   <si>
@@ -190,6 +202,12 @@
     <t>26-aug-26</t>
   </si>
   <si>
+    <t>04-sep-26</t>
+  </si>
+  <si>
+    <t>08-sep-26</t>
+  </si>
+  <si>
     <t>68.57% (24 de 35)</t>
   </si>
   <si>
@@ -226,6 +244,12 @@
     <t>82.05% (32 de 39)</t>
   </si>
   <si>
+    <t>76.92% (40 de 52)</t>
+  </si>
+  <si>
+    <t>76.92% (20 de 26)</t>
+  </si>
+  <si>
     <t>66.67% (16 de 24)</t>
   </si>
   <si>
@@ -274,6 +298,12 @@
     <t>50.00% (16 de 32)</t>
   </si>
   <si>
+    <t>37.50% (15 de 40)</t>
+  </si>
+  <si>
+    <t>75.00% (15 de 20)</t>
+  </si>
+  <si>
     <t>31.43% (11 de 35)</t>
   </si>
   <si>
@@ -308,6 +338,12 @@
   </si>
   <si>
     <t>17.95% (7 de 39)</t>
+  </si>
+  <si>
+    <t>23.08% (12 de 52)</t>
+  </si>
+  <si>
+    <t>23.08% (6 de 26)</t>
   </si>
 </sst>
 </file>
@@ -639,7 +675,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -673,19 +709,19 @@
         <v>2026</v>
       </c>
       <c r="C2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E2" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="F2" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="G2" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -696,19 +732,19 @@
         <v>2026</v>
       </c>
       <c r="C3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D3" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E3" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="F3" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="G3" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -719,19 +755,19 @@
         <v>2026</v>
       </c>
       <c r="C4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E4" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="F4" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="G4" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -742,19 +778,19 @@
         <v>2026</v>
       </c>
       <c r="C5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D5" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E5" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="F5" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="G5" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -765,19 +801,19 @@
         <v>2026</v>
       </c>
       <c r="C6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D6" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E6" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="F6" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="G6" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -788,19 +824,19 @@
         <v>2026</v>
       </c>
       <c r="C7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D7" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E7" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="F7" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="G7" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -811,19 +847,19 @@
         <v>2026</v>
       </c>
       <c r="C8" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D8" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E8" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="F8" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="G8" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -834,19 +870,19 @@
         <v>2026</v>
       </c>
       <c r="C9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D9" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E9" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="F9" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="G9" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -857,19 +893,19 @@
         <v>2026</v>
       </c>
       <c r="C10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D10" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="E10" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="F10" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="G10" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -880,19 +916,19 @@
         <v>2026</v>
       </c>
       <c r="C11" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D11" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E11" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F11" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="G11" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -903,19 +939,19 @@
         <v>2026</v>
       </c>
       <c r="C12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D12" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="E12" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="F12" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="G12" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -926,19 +962,19 @@
         <v>2026</v>
       </c>
       <c r="C13" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D13" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E13" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="F13" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="G13" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -949,19 +985,19 @@
         <v>2026</v>
       </c>
       <c r="C14" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D14" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E14" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F14" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="G14" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -972,19 +1008,19 @@
         <v>2026</v>
       </c>
       <c r="C15" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D15" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="E15" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="F15" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="G15" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -995,19 +1031,19 @@
         <v>2026</v>
       </c>
       <c r="C16" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D16" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E16" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="F16" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="G16" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -1018,19 +1054,19 @@
         <v>2026</v>
       </c>
       <c r="C17" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D17" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="E17" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="F17" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="G17" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -1041,19 +1077,65 @@
         <v>2026</v>
       </c>
       <c r="C18" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D18" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="E18" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="F18" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="G18" t="s">
-        <v>97</v>
+        <v>107</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19">
+        <v>2026</v>
+      </c>
+      <c r="C19" t="s">
+        <v>43</v>
+      </c>
+      <c r="D19" t="s">
+        <v>62</v>
+      </c>
+      <c r="E19" t="s">
+        <v>76</v>
+      </c>
+      <c r="F19" t="s">
+        <v>94</v>
+      </c>
+      <c r="G19" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20">
+        <v>2026</v>
+      </c>
+      <c r="C20" t="s">
+        <v>44</v>
+      </c>
+      <c r="D20" t="s">
+        <v>63</v>
+      </c>
+      <c r="E20" t="s">
+        <v>77</v>
+      </c>
+      <c r="F20" t="s">
+        <v>95</v>
+      </c>
+      <c r="G20" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>